<commit_message>
Publish Intermediate M02 after technical validation
</commit_message>
<xml_diff>
--- a/downloads/exercises/intermedio-m02-m02-l01-practice-01.xlsx
+++ b/downloads/exercises/intermedio-m02-m02-l01-practice-01.xlsx
@@ -657,7 +657,7 @@
       </x:c>
       <x:c r="B9" s="18"/>
       <x:c r="C9" t="str">
-        <x:v>Ventas[#Data]</x:v>
+        <x:v>Ventas[#Datos]</x:v>
       </x:c>
       <x:c r="D9"/>
     </x:row>
@@ -704,7 +704,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="4" t="str">
-        <x:v>5. Distingue Ventas[Importe], Ventas[#Data] y una referencia de fila actual como [@Importe].</x:v>
+        <x:v>5. Distingue Ventas[Importe], Ventas[#Datos] y una referencia de fila actual como [@Importe].</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>